<commit_message>
updated classwork March 27
</commit_message>
<xml_diff>
--- a/Excel/data.xlsx
+++ b/Excel/data.xlsx
@@ -8,14 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victoriaordonez\Documents\DataAnalytics-2026\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BAD2F87-55A8-4B4B-9908-C62C8837FF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB249D9-052F-4FDB-88C4-80CC94A2FE64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="13824" windowHeight="13776" xr2:uid="{A50F8352-B7F2-417D-987E-05430117CEAB}"/>
+    <workbookView xWindow="8472" yWindow="0" windowWidth="14664" windowHeight="13776" activeTab="2" xr2:uid="{A50F8352-B7F2-417D-987E-05430117CEAB}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dataset 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dataset 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="17" r:id="rId4"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="31">
   <si>
     <t>DataSet</t>
   </si>
@@ -99,6 +104,36 @@
   </si>
   <si>
     <t>Standard Deviation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Track </t>
+  </si>
+  <si>
+    <t>Time Zone</t>
+  </si>
+  <si>
+    <t>App Dev</t>
+  </si>
+  <si>
+    <t>EST</t>
+  </si>
+  <si>
+    <t>Data Analytics</t>
+  </si>
+  <si>
+    <t>CST</t>
+  </si>
+  <si>
+    <t>PST</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Average of Score</t>
   </si>
 </sst>
 </file>
@@ -154,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -212,17 +247,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -232,16 +288,49 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -252,6 +341,198 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="victoria ordonez" refreshedDate="46108.582983912034" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="10" xr:uid="{16EFAB8F-9DD4-4AA9-90F1-CEAFF70DB42C}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A2:B12" sheet="Dataset 1"/>
+  </cacheSource>
+  <cacheFields count="2">
+    <cacheField name="Student" numFmtId="0">
+      <sharedItems count="10">
+        <s v="Student 1"/>
+        <s v="Student 2"/>
+        <s v="Student 3"/>
+        <s v="Student 4"/>
+        <s v="Student 5"/>
+        <s v="Student 6"/>
+        <s v="Student 7"/>
+        <s v="Student 8"/>
+        <s v="Student 9"/>
+        <s v="Student 10"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Score" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="65" maxValue="95"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="10">
+  <r>
+    <x v="0"/>
+    <n v="65"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="75"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="80"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <n v="85"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <n v="90"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <n v="75"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="80"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="95"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <n v="70"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5955AD9A-E938-49AA-B948-9C9623EC3047}" name="PivotTable6" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="A1:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="2">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="11">
+        <item x="0"/>
+        <item x="9"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Score" fld="1" subtotal="average" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="0">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <chartFormats count="3">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="1" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -578,167 +859,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="6" t="s">
+      <c r="B1" s="6"/>
+      <c r="D1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="7"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <f>MAX(B3:B12)</f>
         <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>65</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <f>MIN(B3:B12)</f>
         <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>70</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <f>MAX(B3:B12)-MIN(B3:B12)</f>
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>75</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <f>AVERAGE(B3:B12)</f>
         <v>78.5</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>80</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <f>MEDIAN(B3:B12)</f>
         <v>77.5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>85</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <f>_xlfn.MODE.SNGL(B3:B12)</f>
         <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>90</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="3">
         <f>_xlfn.STDEV.P(B3:B12)</f>
         <v>8.9582364335844584</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>75</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>80</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>95</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>70</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -748,4 +1013,369 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E5FD1B-A946-4DE3-A47B-477CBFEAB182}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.109375" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="F1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="8"/>
+      <c r="H1" s="17"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="1">
+        <f>MAX(B3:B12)</f>
+        <v>95</v>
+      </c>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="13">
+        <v>65</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="1">
+        <f>MIN(B3:B12)</f>
+        <v>65</v>
+      </c>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="13">
+        <v>70</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="1">
+        <f>MAX(B3:B12)-MIN(B3:B12)</f>
+        <v>30</v>
+      </c>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="13">
+        <v>75</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="1">
+        <f>AVERAGE(B3:B12)</f>
+        <v>78.5</v>
+      </c>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="13">
+        <v>80</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="1">
+        <f>MEDIAN(B3:B12)</f>
+        <v>77.5</v>
+      </c>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="13">
+        <v>85</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="1">
+        <f>_xlfn.MODE.SNGL(B3:B12)</f>
+        <v>70</v>
+      </c>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="13">
+        <v>90</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="3">
+        <f>_xlfn.STDEV.P(B3:B12)</f>
+        <v>8.9582364335844584</v>
+      </c>
+      <c r="H8" s="12"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="13">
+        <v>75</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="13">
+        <v>80</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="11"/>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="13">
+        <v>95</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="11"/>
+      <c r="H11" s="12"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="13">
+        <v>70</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="11"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C74895C-4D1D-4BE0-9C31-085161E57189}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="21">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="21">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="21">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="21">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="21">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="21">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="21">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="21">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="21">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="21">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="20">
+        <v>78.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>